<commit_message>
Added submission date to excel file. Also added pagination in case we get more than 500 emails.
</commit_message>
<xml_diff>
--- a/2026_Gift_Contest.xlsx
+++ b/2026_Gift_Contest.xlsx
@@ -413,41 +413,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Submission Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>First Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Last Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Address</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>City/State/Zip</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Requirements</t>
         </is>
@@ -456,35 +461,40 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Thu, 07 May 2026 15:06:20 +0000 (UTC)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>John</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Strack</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>john@looploc.com</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>6315822626</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>john@looploc.com</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Hauppauge, New York  11788</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -493,35 +503,40 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Thu, 07 May 2026 13:20:47 +0000 (UTC)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>Test</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>sean.zaletel@loungelizard.com</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>5164739094</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>sean.zaletel@loungelizard.com</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Holbrook, NY  11741</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -530,35 +545,40 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>Thu, 07 May 2026 13:18:27 +0000 (UTC)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>Timothy</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Braun</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>ken.braun@loungelizard.com</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>6313384887</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>ken.braun@loungelizard.com</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Holbrook, NY  11741</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -567,35 +587,40 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Wed, 06 May 2026 15:21:33 +0000 (UTC)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>Ken</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Braun</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>ken.braun@loungelizard.com</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>6315811000</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>ken.braun@loungelizard.com</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Holbrook, NY  11741</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>1</t>
         </is>

</xml_diff>